<commit_message>
Update TTS config and Excel import flow
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -148,42 +148,57 @@
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
+        <t>Nhóm câu hỏi khách/ops tự điền, ví dụ: Giá bán &amp; khuyến mãi, Chất lượng...</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Câu hỏi thật khách sẽ hỏi trong live. Dùng để rà soát/map intent, không đem TTS.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
         <t>Script cần chuyển thành giọng nói (TTS). BẮT BUỘC.</t>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
+    <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <t>Chọn từ dropdown: gioi_thieu (giới thiệu) hoặc tra_loi (trả lời câu hỏi).</t>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <t>CHỈ khi video_type = tra_loi — chọn loại câu hỏi (ASK_*) từ dropdown.</t>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Chỉ điền khi question_type=ASK_OTHER. Ví dụ: khautrang, combo_quatang.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <t>Đường dẫn local video avatar (không bắt buộc). TRỐNG = dùng video mặc định.</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
+    <comment ref="K1" authorId="0" shapeId="0">
       <text>
         <t>(Hệ không xử lý) — để trống.</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="L1" authorId="0" shapeId="0">
       <text>
         <t>HỆ TỰ ĐIỀN sau khi render xong (đường dẫn local video). Khách để TRỐNG.</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>Chọn từ dropdown: vbee / ausynclab / local. TRỐNG = mặc định.</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <t>Chọn giọng từ dropdown. TRỐNG = giọng mặc định của provider.</t>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>Chọn từ dropdown: vbee / ausynclab / autovoice / local. TRỐNG = mặc định.</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <t>Chọn giọng từ dropdown hoặc nhập voice_name. TRỐNG = giọng mặc định của provider.</t>
       </text>
     </comment>
   </commentList>
@@ -479,20 +494,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -513,40 +531,55 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>question_text</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>subText</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>video_type</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>question_type</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>other_key</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>video_path</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>video_url</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>video_done</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>tts_provider</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>tts_voice</t>
         </is>
@@ -560,26 +593,29 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
         <is>
           <t>Chào cả nhà, hôm nay shop có sản phẩm cực hot!</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>gioi_thieu</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
         <is>
           <t>vbee</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -591,74 +627,100 @@
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
+          <t>Giá bán &amp; Chương trình khuyến mãi</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Giá của sản phẩm này là bao nhiêu?</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Dạ giá chỉ 299k ạ, đang sale cực mạnh!</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>tra_loi</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>ASK_PRICE</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
         <is>
           <t>vbee</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>set kep toc</t>
+          <t>khau trang y te</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Bấm giỏ hàng chốt đơn ngay đi ạ!</t>
+          <t>Thông tin sản phẩm</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>Khẩu trang có dùng được khi đi nắng không?</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Dạ khẩu trang nhà em dùng thoải mái khi đi ngoài trời hằng ngày ạ.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>tra_loi</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>ASK_BUY</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr">
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ASK_OTHER</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>khautrang</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
         <is>
           <t>local</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_lists!$A$2:$A$3</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_lists!$B$2:$B$10</formula1>
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>_lists!$B$2:$B$17</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_lists!$C$2:$C$4</formula1>
+    <dataValidation sqref="M2:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>_lists!$C$2:$C$5</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_lists!$D$2:$D$9</formula1>
     </dataValidation>
   </dataValidations>
@@ -673,7 +735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -750,7 +812,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>autovoice</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -765,6 +827,11 @@
           <t>ASK_STOCK</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>n_hanoi_male_quangquangcao_advertise_vc</t>
@@ -823,6 +890,55 @@
       <c r="B10" t="inlineStr">
         <is>
           <t>ASK_PRODUCT</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ASK_MATERIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ASK_SIZE_FIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ASK_EXPIRY</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ASK_CHILDREN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ASK_COLOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ASK_CHECK</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ASK_OTHER</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update logic render musetalk
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -721,7 +721,7 @@
       <formula1>_lists!$C$2:$C$5</formula1>
     </dataValidation>
     <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_lists!$D$2:$D$9</formula1>
+      <formula1>_lists!$D$2:$D$13</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -892,6 +892,11 @@
           <t>ASK_PRODUCT</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>pv-fdb7a34a-243d-42f2-bbcb-cb78cfd027fa</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
@@ -899,6 +904,11 @@
           <t>ASK_MATERIAL</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>pv-a7e16e7d-81e3-45a7-803c-72e22c7dbdc6</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
@@ -906,11 +916,21 @@
           <t>ASK_SIZE_FIT</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>pv-07ea9d28-97d6-49c9-9d60-7d48dc03d4c9</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
           <t>ASK_EXPIRY</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>pv-9518481c-4d54-445d-a5d7-3db2b4114a0a</t>
         </is>
       </c>
     </row>

</xml_diff>